<commit_message>
production files of production run in sept2024
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_A_DAC/Rev02/BOM/BOM_JLC-UZ_A_DAC(THS)_FR_August_2024.xlsx
+++ b/Project Outputs for UZ_A_DAC/Rev02/BOM/BOM_JLC-UZ_A_DAC(THS)_FR_August_2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ga92wum\git\UltraZohm\PCB\uz_a_dac8831\Project Outputs for UZ_A_DAC\Rev02\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCCAC50-4BDE-41F7-8851-31E305B650C2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2357201-A02D-441D-8346-0DE721E9065F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15090" yWindow="-16130" windowWidth="19350" windowHeight="7560" xr2:uid="{8EB92CD4-8990-4A58-AC57-FDF9BBF21F69}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="329">
   <si>
     <t>Quantity</t>
   </si>
@@ -942,9 +942,6 @@
     <t>C149618</t>
   </si>
   <si>
-    <t>C519510</t>
-  </si>
-  <si>
     <t>C513774</t>
   </si>
   <si>
@@ -967,9 +964,6 @@
   </si>
   <si>
     <t>C398931</t>
-  </si>
-  <si>
-    <t>C88219</t>
   </si>
   <si>
     <t>C465462</t>
@@ -1480,10 +1474,10 @@
         <v>10</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
@@ -1513,8 +1507,8 @@
       <c r="J2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="5" t="s">
-        <v>313</v>
+      <c r="K2" s="6" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
@@ -1576,7 +1570,7 @@
         <v>26</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
@@ -1607,7 +1601,7 @@
         <v>31</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
@@ -1638,7 +1632,7 @@
         <v>36</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
@@ -1669,7 +1663,7 @@
         <v>41</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
@@ -1731,7 +1725,7 @@
         <v>50</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
@@ -1762,7 +1756,7 @@
         <v>55</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
@@ -1855,10 +1849,10 @@
         <v>71</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="N13" s="13" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
@@ -1921,10 +1915,10 @@
         <v>77</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="N15" s="1" t="s">
         <v>301</v>
@@ -2111,10 +2105,10 @@
         <v>103</v>
       </c>
       <c r="K21" s="12" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="L21" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="N21" s="8" t="s">
         <v>293</v>
@@ -2364,7 +2358,7 @@
         <v>145</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.35">
@@ -2395,7 +2389,7 @@
         <v>149</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.35">
@@ -2426,7 +2420,7 @@
         <v>153</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.35">
@@ -2519,7 +2513,7 @@
         <v>164</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.35">
@@ -2767,7 +2761,7 @@
         <v>191</v>
       </c>
       <c r="K42" s="7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.35">
@@ -2798,10 +2792,10 @@
         <v>194</v>
       </c>
       <c r="K43" s="9" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="L43" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="N43" s="8" t="s">
         <v>280</v>
@@ -2866,7 +2860,7 @@
         <v>201</v>
       </c>
       <c r="K45" s="7" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.35">
@@ -2897,10 +2891,10 @@
         <v>205</v>
       </c>
       <c r="K46" s="9" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="L46" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="N46" s="8" t="s">
         <v>279</v>
@@ -3255,10 +3249,10 @@
         <v>256</v>
       </c>
       <c r="K58" s="9" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="L58" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="N58" s="8" t="s">
         <v>267</v>

</xml_diff>